<commit_message>
updated viz and transformed data
</commit_message>
<xml_diff>
--- a/Extracted_data_analysis/global/Output-Transformed_data/summary_split_counts_question_1_3.xlsx
+++ b/Extracted_data_analysis/global/Output-Transformed_data/summary_split_counts_question_1_3.xlsx
@@ -8,7 +8,7 @@
   <sheets>
     <sheet name="meso_substrate" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="habit" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="meso_spatial" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="environmentalPosition" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="observationalORexperimental" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="taxonomicTargetLevel" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="indicators" sheetId="6" state="visible" r:id="rId6"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="83">
   <si>
     <t xml:space="preserve">meso_substrate</t>
   </si>
@@ -54,10 +54,19 @@
     <t xml:space="preserve">vagile</t>
   </si>
   <si>
-    <t xml:space="preserve">meso_spatial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">x</t>
+    <t xml:space="preserve">environmentalPosition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">epi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">endo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pelagic</t>
   </si>
   <si>
     <t xml:space="preserve">observationalORexperimental</t>
@@ -120,6 +129,9 @@
     <t xml:space="preserve">surv</t>
   </si>
   <si>
+    <t xml:space="preserve">geneticSequences</t>
+  </si>
+  <si>
     <t xml:space="preserve">Density</t>
   </si>
   <si>
@@ -159,67 +171,67 @@
     <t xml:space="preserve">func</t>
   </si>
   <si>
+    <t xml:space="preserve">sample</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">taxonomy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">disease</t>
+  </si>
+  <si>
+    <t xml:space="preserve">economicValue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ecoser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">orientation</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Diversity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fecundity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">collectedDataType</t>
+  </si>
+  <si>
+    <t xml:space="preserve">photo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">video</t>
+  </si>
+  <si>
+    <t xml:space="preserve">specimen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sediment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">water</t>
+  </si>
+  <si>
+    <t xml:space="preserve">molecularAnalyses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no</t>
+  </si>
+  <si>
+    <t xml:space="preserve">genotyping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes</t>
+  </si>
+  <si>
     <t xml:space="preserve">phylo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sample</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sex</t>
-  </si>
-  <si>
-    <t xml:space="preserve">taxonomy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">disease</t>
-  </si>
-  <si>
-    <t xml:space="preserve">economicValue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ecoser</t>
-  </si>
-  <si>
-    <t xml:space="preserve">orientation</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Diversity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fecundity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">collectedDataType</t>
-  </si>
-  <si>
-    <t xml:space="preserve">photo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">video</t>
-  </si>
-  <si>
-    <t xml:space="preserve">specimen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sediment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">visual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">water</t>
-  </si>
-  <si>
-    <t xml:space="preserve">molecularAnalyses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">no</t>
-  </si>
-  <si>
-    <t xml:space="preserve">genotyping</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yes</t>
   </si>
   <si>
     <t xml:space="preserve">phylogenetic</t>
@@ -732,10 +744,54 @@
         <v>12</v>
       </c>
       <c r="B2" t="n">
-        <v>32</v>
+        <v>117</v>
       </c>
       <c r="C2" t="n">
-        <v>74.42</v>
+        <v>11.77</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="n">
+        <v>961</v>
+      </c>
+      <c r="C3" t="n">
+        <v>96.68</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="n">
+        <v>70</v>
+      </c>
+      <c r="C4" t="n">
+        <v>7.04</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>
@@ -751,7 +807,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -762,7 +818,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B2" t="n">
         <v>956</v>
@@ -773,7 +829,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B3" t="n">
         <v>97</v>
@@ -795,7 +851,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -806,7 +862,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B2" t="n">
         <v>386</v>
@@ -817,7 +873,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B3" t="n">
         <v>332</v>
@@ -828,7 +884,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B4" t="n">
         <v>197</v>
@@ -839,7 +895,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B5" t="n">
         <v>200</v>
@@ -861,7 +917,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -872,7 +928,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B2" t="n">
         <v>344</v>
@@ -883,7 +939,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B3" t="n">
         <v>309</v>
@@ -894,7 +950,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B4" t="n">
         <v>455</v>
@@ -905,7 +961,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B5" t="n">
         <v>180</v>
@@ -916,7 +972,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B6" t="n">
         <v>242</v>
@@ -927,7 +983,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B7" t="n">
         <v>6</v>
@@ -938,7 +994,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B8" t="n">
         <v>218</v>
@@ -949,7 +1005,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B9" t="n">
         <v>121</v>
@@ -960,7 +1016,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B10" t="n">
         <v>68</v>
@@ -971,7 +1027,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B11" t="n">
         <v>16</v>
@@ -982,7 +1038,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B12" t="n">
         <v>28</v>
@@ -993,161 +1049,161 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B13" t="n">
-        <v>219</v>
+        <v>159</v>
       </c>
       <c r="C13" t="n">
-        <v>22.03</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B14" t="n">
-        <v>42</v>
+        <v>219</v>
       </c>
       <c r="C14" t="n">
-        <v>4.23</v>
+        <v>22.03</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B15" t="n">
-        <v>89</v>
+        <v>42</v>
       </c>
       <c r="C15" t="n">
-        <v>8.95</v>
+        <v>4.23</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B16" t="n">
-        <v>127</v>
+        <v>89</v>
       </c>
       <c r="C16" t="n">
-        <v>12.78</v>
+        <v>8.95</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B17" t="n">
-        <v>64</v>
+        <v>127</v>
       </c>
       <c r="C17" t="n">
-        <v>6.44</v>
+        <v>12.78</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B18" t="n">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="C18" t="n">
-        <v>5.53</v>
+        <v>6.44</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B19" t="n">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="C19" t="n">
-        <v>3.92</v>
+        <v>5.53</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B20" t="n">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="C20" t="n">
-        <v>6.34</v>
+        <v>3.92</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>63</v>
       </c>
       <c r="C21" t="n">
-        <v>0.1</v>
+        <v>6.34</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B22" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>2.72</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B23" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C23" t="n">
-        <v>2.41</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B24" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C24" t="n">
-        <v>2.52</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B25" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C25" t="n">
-        <v>2.01</v>
+        <v>2.52</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B26" t="n">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C26" t="n">
-        <v>5.13</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B27" t="n">
         <v>1</v>
@@ -1158,7 +1214,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B28" t="n">
         <v>22</v>
@@ -1169,7 +1225,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B29" t="n">
         <v>1</v>
@@ -1180,7 +1236,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B30" t="n">
         <v>7</v>
@@ -1191,7 +1247,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B31" t="n">
         <v>1</v>
@@ -1202,7 +1258,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B32" t="n">
         <v>3</v>
@@ -1213,7 +1269,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B33" t="n">
         <v>1</v>
@@ -1224,7 +1280,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B34" t="n">
         <v>1</v>
@@ -1235,7 +1291,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B35" t="n">
         <v>1</v>
@@ -1257,7 +1313,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -1268,7 +1324,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B2" t="n">
         <v>347</v>
@@ -1279,7 +1335,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B3" t="n">
         <v>421</v>
@@ -1290,18 +1346,18 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B4" t="n">
-        <v>309</v>
+        <v>557</v>
       </c>
       <c r="C4" t="n">
-        <v>31.09</v>
+        <v>56.04</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B5" t="n">
         <v>44</v>
@@ -1312,7 +1368,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B6" t="n">
         <v>124</v>
@@ -1323,34 +1379,23 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="B7" t="n">
-        <v>248</v>
+        <v>25</v>
       </c>
       <c r="C7" t="n">
-        <v>24.95</v>
+        <v>2.52</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>62</v>
+        <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>2.52</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -1367,7 +1412,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -1378,7 +1423,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B2" t="n">
         <v>915</v>
@@ -1389,7 +1434,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B3" t="n">
         <v>63</v>
@@ -1400,7 +1445,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B4" t="n">
         <v>6</v>
@@ -1422,7 +1467,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="B6" t="n">
         <v>42</v>
@@ -1433,7 +1478,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B7" t="n">
         <v>9</v>
@@ -1444,7 +1489,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B8" t="n">
         <v>21</v>
@@ -1455,7 +1500,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B9" t="n">
         <v>18</v>
@@ -1466,7 +1511,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B10" t="n">
         <v>40</v>
@@ -1477,7 +1522,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B11" t="n">
         <v>3</v>
@@ -1488,7 +1533,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B12" t="n">
         <v>5</v>
@@ -1499,7 +1544,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B13" t="n">
         <v>1</v>
@@ -1510,7 +1555,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B14" t="n">
         <v>11</v>
@@ -1521,7 +1566,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B15" t="n">
         <v>1</v>
@@ -1532,7 +1577,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B16" t="n">
         <v>1</v>
@@ -1543,7 +1588,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B17" t="n">
         <v>1</v>
@@ -1554,7 +1599,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B18" t="n">
         <v>2</v>

</xml_diff>